<commit_message>
Fontes 5–7: GPS BRT, nível de rios ANA e queimadas INPE
BRT entra no job quente (851 veículos/snapshot, campos ricos no extra).
Rios ANA: 4 estações urbanas com coords do HidroInventario, parser tolera
estação muda (serviço frágil). INPE: filtro de município em duas etapas
(bbox no parser + exigir_bairro na gravação) e dedup natural de evento
pontual por (tipo, inicio, h3). Planilha de fontes atualizada.

Claude-Session: https://claude.ai/code/session_01L58aWXsvNNs8RhGKvEKeZA
</commit_message>
<xml_diff>
--- a/fontes.xlsx
+++ b/fontes.xlsx
@@ -954,9 +954,9 @@
           <t>Queimadas INPE</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>🔜 planejada</t>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>✅ NO AR</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -989,7 +989,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>CSV não filtra município: usa nosso point-in-polygon de bairros (já pronto)</t>
+          <t>Filtro do município em 2 etapas (bbox no parser + bairro na gravação); lê os 3 arquivos mais novos com dedup. No ar desde 2026-08-06</t>
         </is>
       </c>
     </row>
@@ -1004,9 +1004,9 @@
           <t>Nível de rios (ANA/INEA)</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>🔜 planejada</t>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>✅ NO AR</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Complementa pluviômetro no painel de enchente; estações 59305027/35/55/71</t>
+          <t>Serviço frágil (parser tolera estação muda — Acari sem dado em 06/08); coords do HidroInventario. No ar desde 2026-08-06</t>
         </is>
       </c>
     </row>
@@ -1104,9 +1104,9 @@
           <t>GPS BRT</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>🔜 planejada</t>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>✅ NO AR</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Formato diferente do SPPO: parser separado</t>
+          <t>Formato diferente do SPPO: parser separado. No ar desde 2026-08-06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
GTFS, snapshot da cidade, radar (blobs) e previsão Open-Meteo
- GTFS da SMTR carregado via COPY (492 rotas, 1M stop_times); 96% das
  linhas do GPS casam com o planejado — Tese 3 destravada.
- Job snapshot_cidade a cada 15 min: fotografia resumida pro replay.
- Radar do Sumaré: armazém de blobs (disco em dev, R2 decidido pra prod)
  com manifesto e dedup por Last-Modified; ./dados montado no compose.
- Previsão como 4ª natureza (decisão A de 2026-08-06): tabela previsao
  guarda todas as rodadas com emitida_em; painel lê vw_previsao_atual.
  Fontes previsao_tempo (5 zonas) e previsao_mar (2 pontos), cron 3h.

Claude-Session: https://claude.ai/code/session_01L58aWXsvNNs8RhGKvEKeZA
</commit_message>
<xml_diff>
--- a/fontes.xlsx
+++ b/fontes.xlsx
@@ -56,12 +56,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00EEEEEE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EEEEEE"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -608,9 +608,9 @@
           <t>Radar do Sumaré</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>🔜 planejada</t>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>✅ NO AR</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -643,7 +643,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Blob fora do banco (disco/R2) com manifesto; retenção 1 ano (~1.6 GB) por DEC</t>
+          <t>Blob no armazém (disco em dev; R2 decidido pra prod) + manifesto; retenção 1 ano por DEC. Análise de pixels: v2. No ar desde 2026-08-06</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
           <t>Web Sirene / Defesa Civil</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>❓ investigar</t>
         </is>
@@ -758,7 +758,7 @@
           <t>CEMADEN — alertas</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>❓ investigar</t>
         </is>
@@ -808,14 +808,14 @@
           <t>Open-Meteo — previsão</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>🔜 planejada</t>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>✅ NO AR</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>medicao</t>
+          <t>previsao (4ª natureza)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>1 h</t>
+          <t>3 h</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
@@ -843,7 +843,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Substitui o papel do INMET (que morreu)</t>
+          <t>Decisão A 2026-08-06: TODAS as rodadas guardadas (emitida_em na chave); painel lê vw_previsao_atual. 5 pontos, um por zona. No ar desde 2026-08-06</t>
         </is>
       </c>
     </row>
@@ -858,14 +858,14 @@
           <t>Open-Meteo — Marine</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>🔜 planejada</t>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>✅ NO AR</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>medicao</t>
+          <t>previsao (4ª natureza)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>1 h</t>
+          <t>3 h</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
@@ -891,7 +891,11 @@
           <t>não</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>2 pontos no litoral (Copacabana e Barra). No ar desde 2026-08-06</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -904,7 +908,7 @@
           <t>Tábua de marés (CHM/Marinha)</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>🔜 planejada (estática)</t>
         </is>
@@ -1154,9 +1158,9 @@
           <t>GTFS estático</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>🔜 planejada</t>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>✅ CARREGADA (seed)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1189,7 +1193,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Base do planejado × realizado e do detector de linha parada</t>
+          <t>Carregado 2026-08-06: 492 rotas, 17.4k viagens, 1M stop_times; 96% das linhas do GPS casam com o GTFS</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1208,7 @@
           <t>api.mobilidade.rio (ETA)</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>🔜 avaliar</t>
         </is>
@@ -1254,7 +1258,7 @@
           <t>MetrôRio — status</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>🔜 planejada (frágil)</t>
         </is>
@@ -1304,7 +1308,7 @@
           <t>Aviões (adsb.lol)</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>🔜 planejada</t>
         </is>
@@ -1354,7 +1358,7 @@
           <t>Aviões (OpenSky)</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>🔜 fallback</t>
         </is>
@@ -1454,7 +1458,7 @@
           <t>Trânsito (TomTom)</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>🔜 planejada (chave OK)</t>
         </is>
@@ -1504,7 +1508,7 @@
           <t>ANAC VRA (voos realizados)</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>🔜 planejada</t>
         </is>
@@ -1604,7 +1608,7 @@
           <t>ISP-RJ (estatísticas)</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>🔜 planejada</t>
         </is>
@@ -1654,7 +1658,7 @@
           <t>GeoRio — risco geológico</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>🔜 planejada (estática)</t>
         </is>
@@ -1854,7 +1858,7 @@
           <t>IBGE — população</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>🔜 planejada</t>
         </is>
@@ -1904,7 +1908,7 @@
           <t>Balneabilidade INEA</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>🔜 planejada</t>
         </is>
@@ -2054,7 +2058,7 @@
           <t>Agenda de jogos (TheSportsDB)</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t>🔜 planejada</t>
         </is>
@@ -2104,7 +2108,7 @@
           <t>Águas do Rio — comunicados</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>🔜 planejada</t>
         </is>
@@ -2154,7 +2158,7 @@
           <t>Saúde SMS (vigilância)</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>❓ avaliar</t>
         </is>
@@ -2204,7 +2208,7 @@
           <t>Drenagem / SABREN (estáticas)</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr">
         <is>
           <t>🔜 planejada (estática)</t>
         </is>
@@ -2300,7 +2304,7 @@
           <t>Diário Oficial do Município</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="C37" s="5" t="inlineStr">
         <is>
           <t>🔜 planejada</t>
         </is>

</xml_diff>

<commit_message>
Fontes 13–17: aviões, MetrôRio, jogos, Águas do Rio e TomTom
- ceu_adsb: aeronaves em raio de 40 nm, seen>60s descartado, job quente.
- metro_rio: token Bearer re-extraído do JS do site a cada coleta; só
  status anormal vira evento vigente por linha (novo `encerrar` no
  contrato fecha o evento quando normaliza; vigência agora compara
  severidade+título, não inicio).
- jogos (TheSportsDB): 4 grandes, filtro por estádio DA CIDADE com
  coordenada real — jogo vira evento com pino e janela de 2h30.
- aguas_rio: comunicados (categoria 449 do WP), HTML limpo.
- transito_tomtom: 12 corredores propostos, amostragem pico 15/15min e
  fora-de-pico 1/h (~17,3k req/mês no free tier de 20k).
Cards Céu, Cidade viva (parametrizado) e metrô no Mobilidade agora reais.

Claude-Session: https://claude.ai/code/session_01L58aWXsvNNs8RhGKvEKeZA
</commit_message>
<xml_diff>
--- a/fontes.xlsx
+++ b/fontes.xlsx
@@ -1258,9 +1258,9 @@
           <t>MetrôRio — status</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>🔜 planejada (frágil)</t>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>✅ NO AR (frágil)</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1293,7 +1293,7 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Token de terceiro embutido: monitorar quebra</t>
+          <t>Token re-extraído do JS do site a cada coleta (resiliente à rotação). Só anormal vira evento; normal encerra. No ar desde 2026-08-06</t>
         </is>
       </c>
     </row>
@@ -1308,9 +1308,9 @@
           <t>Aviões (adsb.lol)</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>🔜 planejada</t>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>✅ NO AR</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Usar campo `seen` pra descartar posição velha</t>
+          <t>seen&gt;60s descartado; céu vazio é sucesso. No ar desde 2026-08-06</t>
         </is>
       </c>
     </row>
@@ -1458,9 +1458,9 @@
           <t>Trânsito (TomTom)</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>🔜 planejada (chave OK)</t>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>✅ NO AR (amostrado)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Estratégia da DEC: camada base = velocidade derivada do NOSSO GPS de ônibus; TomTom só amostra corredores</t>
+          <t>12 corredores propostos (Luciano pode editar em transito_tomtom.py); pico = 15/15min, fora = 1/h ≈ 17,3k req/mês no free tier de 20k. No ar desde 2026-08-06</t>
         </is>
       </c>
     </row>
@@ -2058,9 +2058,9 @@
           <t>Agenda de jogos (TheSportsDB)</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>🔜 planejada</t>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>✅ NO AR</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -2093,7 +2093,7 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>Filtrar venue no cliente (endpoint por venue é premium); shows não esportivos não têm fonte</t>
+          <t>Venues do Rio com coordenada real (jogo vira evento com pino). No ar desde 2026-08-06</t>
         </is>
       </c>
     </row>
@@ -2108,9 +2108,9 @@
           <t>Águas do Rio — comunicados</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>🔜 planejada</t>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>✅ NO AR</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>Baixa frequência; contexto</t>
+          <t>Categoria 449 (comunicados); atende a metropolitana inteira — sem filtro geográfico na v1. No ar desde 2026-08-06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fontes 18–19: Diário Oficial e ISP-RJ (backfill 2003–2026)
- diario_oficial: edições do dia e da véspera como blob PDF no R2 com
  manifesto; pula edição já armazenada (evita rebaixar ~30 MB/rodada);
  tolerância de 4 dias (fim de semana sem edição é normal).
- isp_rj: CSV mensal por CISP filtrado pra Capital e somado por mês —
  primeira coleta backfillou 282 meses × 6 métricas (1.692 medições,
  jan/2003–jun/2026): a primeira série histórica longa do banco.
- Cron ganhou faixas diária/semanal; investigações encerradas e
  documentadas na planilha: CEMADEN descartada (rede degradada no
  município: 11/30 estações vivas, acumulados vazios), sirenes Defesa
  Civil bloqueada por token (caminho institucional).

Claude-Session: https://claude.ai/code/session_01L58aWXsvNNs8RhGKvEKeZA
</commit_message>
<xml_diff>
--- a/fontes.xlsx
+++ b/fontes.xlsx
@@ -56,17 +56,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EEEEEE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9D2E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEEEEE"/>
       </patternFill>
     </fill>
     <fill>
@@ -708,9 +708,9 @@
           <t>Web Sirene / Defesa Civil</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>❓ investigar</t>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>⛔ bloqueada (token)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Investigar acesso direto ao pgeo3</t>
+          <t>Confirmado 2026-08-06: pgeo3 direto também exige token (ArcGIS 499). Caminho = contato institucional com a Defesa Civil</t>
         </is>
       </c>
     </row>
@@ -755,12 +755,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>CEMADEN — alertas</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>❓ investigar</t>
+          <t>CEMADEN — pluviômetros</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>⛔ investigada e descartada</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -775,12 +775,12 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>www2.cemaden.gov.br — sem API REST óbvia; investigar XHR do mapa interativo</t>
+          <t>resources.cemaden.gov.br/graficos/interativo/getJson2.php?uf=RJ (achado 2026-08-06)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>15 min (proposta)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
@@ -793,7 +793,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>URL do plano original estava morta; download oficial é por e-mail</t>
+          <t>Endpoint fácil, MAS rede degradada no município: só 11/30 estações com leitura em 24h e acumulados todos vazios. Alerta Rio cobre melhor; reavaliar se a rede reviver</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
           <t>Tábua de marés (CHM/Marinha)</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>🔜 planejada (estática)</t>
         </is>
@@ -1208,7 +1208,7 @@
           <t>api.mobilidade.rio (ETA)</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>🔜 avaliar</t>
         </is>
@@ -1358,7 +1358,7 @@
           <t>Aviões (OpenSky)</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>🔜 fallback</t>
         </is>
@@ -1408,7 +1408,7 @@
           <t>Navios (aisstream.io)</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>⏸️ instável (stream mudo)</t>
         </is>
@@ -1508,7 +1508,7 @@
           <t>ANAC VRA (voos realizados)</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>🔜 planejada</t>
         </is>
@@ -1558,7 +1558,7 @@
           <t>Fogo Cruzado</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>⏸️ POR ÚLTIMO (DEC)</t>
         </is>
@@ -1608,9 +1608,9 @@
           <t>ISP-RJ (estatísticas)</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>🔜 planejada</t>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>✅ NO AR + BACKFILL</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Usar host COM www (sem www o TLS falha); alimenta normalização por 100 mil</t>
+          <t>Host COM www. Capital agregada por mês: 282 meses (2003–2026) × 6 métricas backfillados na 1ª coleta. No ar desde 2026-08-06</t>
         </is>
       </c>
     </row>
@@ -1658,7 +1658,7 @@
           <t>GeoRio — risco geológico</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>🔜 planejada (estática)</t>
         </is>
@@ -1708,7 +1708,7 @@
           <t>Chamados 1746</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>⏸️ fase 2 (DEC)</t>
         </is>
@@ -1858,7 +1858,7 @@
           <t>IBGE — população</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>🔜 planejada</t>
         </is>
@@ -1908,7 +1908,7 @@
           <t>Balneabilidade INEA</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>🔜 planejada</t>
         </is>
@@ -1958,7 +1958,7 @@
           <t>Notícias RSS (G1/Extra/O Dia/Google News)</t>
         </is>
       </c>
-      <c r="C30" s="6" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>⏸️ v2 (pacote LLM)</t>
         </is>
@@ -2008,7 +2008,7 @@
           <t>Bluesky do COR</t>
         </is>
       </c>
-      <c r="C31" s="6" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>⏸️ v2 (pacote LLM)</t>
         </is>
@@ -2158,7 +2158,7 @@
           <t>Saúde SMS (vigilância)</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr">
         <is>
           <t>❓ avaliar</t>
         </is>
@@ -2208,7 +2208,7 @@
           <t>Drenagem / SABREN (estáticas)</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>🔜 planejada (estática)</t>
         </is>
@@ -2304,9 +2304,9 @@
           <t>Diário Oficial do Município</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>🔜 planejada</t>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>✅ NO AR</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>diário</t>
+          <t>6 h (edições saem ao longo do dia)</t>
         </is>
       </c>
       <c r="H37" s="2" t="n">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>Upgrade sobre o plano (que supunha PDF cru)</t>
+          <t>PDF vira blob no R2 com manifesto; fim de semana sem edição é normal. No ar desde 2026-08-06</t>
         </is>
       </c>
     </row>
@@ -2354,7 +2354,7 @@
           <t>Relatórios Fogo Cruzado / boletins ISP</t>
         </is>
       </c>
-      <c r="C38" s="6" t="inlineStr">
+      <c r="C38" s="5" t="inlineStr">
         <is>
           <t>⏸️ fase 3</t>
         </is>

</xml_diff>

<commit_message>
Fonte 20: Fogo Cruzado — a "por último" entra no ar, com backfill 2016+
Autorização concedida pelo Instituto em 2026-08-06. Login JWT por rodada
(credenciais FOGO_CRUZADO_USER/PASSWORD via alias no config), filtro
estado RJ + cidade Rio (UUIDs descobertos ao vivo), janela rolante de 3
dias com dedup. Conforme a DEC de exibição: pino exato, sem visivel_apos;
severidade 3 sem vítima / 4 com vítima; payload completo (motivo, ação
policial, mortos/feridos, recortes). Seed de backfill paginado desde
2016 (28,6 mil ocorrências) rodando. Card Segurança real: ocorrências
24h do Fogo Cruzado + última letalidade mensal do ISP.

Claude-Session: https://claude.ai/code/session_01L58aWXsvNNs8RhGKvEKeZA
</commit_message>
<xml_diff>
--- a/fontes.xlsx
+++ b/fontes.xlsx
@@ -1558,9 +1558,9 @@
           <t>Fogo Cruzado</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>⏸️ POR ÚLTIMO (DEC)</t>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>✅ NO AR + BACKFILL</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1580,7 +1580,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>5 min (quando autorizado)</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="H22" s="2" t="n">
@@ -1588,12 +1588,12 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>SIM (autorização)</t>
+          <t>SIM (no .env)</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Pedido de autorização só com estrutura demonstrável; termos deles exigem crédito (rotulagem já é requisito)</t>
+          <t>Autorização concedida em 2026-08-06; login JWT (credenciais no .env), pino exato por DEC, severidade 3/4 por vítimas, backfill 2016+ (28,6 mil ocorrências). Crédito obrigatório nos painéis</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fontes.xlsx atualizada e aba de data, pra ela não parecer atual sem ser
A planilha estava congelada em 01:57 de 2026-08-07, antes de tudo que a sessão
mudou — e planilha desatualizada com cara de atual é o mesmo defeito que a gente
passou o dia tirando da interface.

Atualizado em cima (as descrições vieram do catálogo do vault e não saem do
código, então regenerar do zero perderia conteúdo): SPPO com o schema GTFS novo,
a pegadinha do Z mentiroso e o backfill; COR com o `id` que não é o estágio;
MetrôRio marcado como fora em produção pelo 403 do datacenter; balneabilidade
registrando que a ausência agora é declarada no card.

Linha nova pro detector de linha parada — é derivado, não fonte externa, mas
aparece na página pública de status, então precisa estar aqui.

Aba "Atualização" com data e resumo do que mudou: sem isso não há como saber se
a planilha é de hoje ou de três semanas atrás.

Claude-Session: https://claude.ai/code/session_017njQDdLcvLKzJzig7fyLXD
</commit_message>
<xml_diff>
--- a/fontes.xlsx
+++ b/fontes.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Fontes" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Cadências" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Descartadas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fontes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cadências" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Descartadas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atualização" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Fontes'!$A$1:$J$38</definedName>
@@ -92,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -113,6 +114,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -480,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -693,7 +697,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Domínio interno frágil; fallback = raspar cor.rio. Mudança de estágio fecha o evento anterior e abre outro</t>
+          <t>Domínio interno frágil; fallback = raspar cor.rio. Mudança de estágio fecha o evento anterior e abre outro. PEGADINHA: o campo `id` NÃO é o estágio (em 2026-08-06 ficou 1 com o texto "Estágio 2"). Quem manda é o texto; a cor corrobora sem reprovar. Crosscheck antigo derrubou a fonte por um dia — ver DEC - Crosscheck de fonte só reprova o que invalida o dado</t>
         </is>
       </c>
     </row>
@@ -1060,7 +1064,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>✅ NO AR</t>
+          <t>✅ NO AR + BACKFILL</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1070,12 +1074,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Posição, velocidade, linha e ordem de ~6 mil ônibus (~15.5k registros/2 min)</t>
+          <t>Posição, velocidade, sentido, direção e a VIAGEM (trip_id/shape_id) de ~4 mil ônibus (~20k registros por janela de 3 min)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>REST dados.mobilidade.rio/gps/sppo com janela dataInicial/dataFinal OBRIGATÓRIA em hora local</t>
+          <t>REST dados.mobilidade.rio/gps/sppo com janela dataInicial/dataFinal OBRIGATÓRIA em hora local (sem ela, HTTP 500). Janelas passadas funcionam: backfill até ~30 h</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1093,7 +1097,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Lat/lon com vírgula; datahora em epoch ms UTC; janelas se sobrepõem (dedup por PK)</t>
+          <t>SCHEMA TROCADO PELA SMTR em 2026-08-07: era ordem/linha/datahora(epoch ms)/lat-lon com vírgula; virou id_veiculo/servico/datetime(ISO)/floats + campos GTFS. 97% dos trip_id casam com a gtfs_trips. PEGADINHA: o sufixo Z do datetime é MENTIRA — é hora local do Rio; sem reetiquetar, tudo entra 3 h no passado em silêncio. route_id vem nulo em 100%. Janelas se sobrepõem (dedup por PK). Backfill: python -m riolive.semente.gps_sppo</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1264,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>✅ NO AR (frágil)</t>
+          <t>⛔ FORA em produção (403)</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1293,7 +1297,7 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Token re-extraído do JS do site a cada coleta (resiliente à rotação). Só anormal vira evento; normal encerra. No ar desde 2026-08-06</t>
+          <t>Token re-extraído do JS do site a cada coleta (resiliente à rotação). Só anormal vira evento; normal encerra. BLOQUEIO: a API devolve HTTP 403 pro IP do datacenter (Contabo) — funciona do WSL. Precisa proxy/outro IP; é decisão de infra, não código</t>
         </is>
       </c>
     </row>
@@ -1943,7 +1947,7 @@
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>TLS sem cadeia intermediária: embutir CA no cliente</t>
+          <t>TLS sem cadeia intermediária: embutir CA no cliente. Enquanto não entra, o card de Mar exibe "—" nos contadores de praia COM o motivo, em vez de número inventado (DEC - Interface não afirma o que não mediu)</t>
         </is>
       </c>
     </row>
@@ -2388,6 +2392,56 @@
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>B · Mobilidade</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Detector de linha parada (DERIVADO)</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>✅ NO AR</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>evento (vigente)</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Linha planejada agora no GTFS sem nenhum veículo com GPS há 40+ min — a tese 3 do produto</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Interno: cruza gtfs_trips/frequencies com posicao. Não é fonte externa, mas aparece na página de status</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>NUNCA roda sem gps_confiavel() (20+ min online e 1.500 ônibus transmitindo) — trava aprendida com 111 falsos positivos. Reporta a própria saúde desde 2026-08-07: online quando avalia, degradada quando espera o GPS. Primeiro evento real: linha SPA613 em 2026-08-07</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:J38"/>
@@ -2724,4 +2778,46 @@
   <autoFilter ref="A1:B13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Atualizada em</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>O que mudou</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>SPPO: schema novo (GTFS) + pegadinha do Z + backfill de posições. COR: id não é o estágio, fonte de volta ao ar. MetrôRio: 403 pro IP do datacenter, fora em produção. Detector de linha parada entrou como linha própria (derivado, aparece no status). Balneabilidade: ausência declarada no card de Mar.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>